<commit_message>
Update soccer trades 2026-08-03 23:03:36 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,92 +531,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>70.81</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.2975</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19516436</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,92 +635,84 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1.43</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.4512</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19516436</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,110 +739,334 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.2975</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785703082</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>3.361345</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-04 03:04:00 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,7 +542,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1785807147</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,15 +643,19 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0525</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -659,7 +663,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1785805367</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>28.761905</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,92 +747,84 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>70.81</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1.2975</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>L19516436</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,92 +851,84 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1.43</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1.4512</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>L19516436</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,110 +955,334 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.2975</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785703082</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>3.361345</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 12:01:21 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4125</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -578,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785807147</t>
+          <t>1786015629</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>19.345455</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,94 +651,86 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1.51</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.0525</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Alverca</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>FC Porto vs Alverca</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FC Porto</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Alverca</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19516476</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785805367</t>
+          <t>1785807147</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>28.761905</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,15 +755,19 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0525</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -771,7 +775,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -779,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1785805367</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>28.761905</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -862,7 +870,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>70.81</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -928,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,92 +963,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1.2975</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>L19516436</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.2975</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1097,32 +1097,32 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785703082</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>3.361345</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,110 +1179,222 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 15:01:32 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
+          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>1.025</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4125</t>
+          <t>1.0513</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786015629</t>
+          <t>1786025695</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>19.345455</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,23 +643,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4125</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -667,7 +671,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -690,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785807147</t>
+          <t>1786015629</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>19.345455</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,19 +763,15 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.0525</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -775,11 +779,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Alverca</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785805367</t>
+          <t>1785807147</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>28.761905</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -867,15 +867,19 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0525</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -883,7 +887,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -891,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1785805367</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>28.761905</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -974,7 +982,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>70.81</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1040,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,27 +1075,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2975</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1095,11 +1099,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,12 +1179,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1194,12 +1194,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.2975</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1209,32 +1209,32 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785703082</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>3.361345</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,110 +1291,222 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 21:02:05 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
+          <t>0xeb3ffa21a81bad64e1c57daa8b3b700ccd2e0a139717709a792ed1a5fe326ca8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.0513</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786025695</t>
+          <t>1786049713</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>11.301587</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
+          <t>0xcbddf823e635f74877809e664d307d69fbe07274867c3fdd6f6b327d9b61cfd2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,19 +651,15 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>165.96</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4125</t>
+          <t>1.4875</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -671,11 +667,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -683,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Vitoria Guimaraes vs FC Arouca</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>FC Arouca</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x1952e4e0eea3adef3eef21ecd14324031f0ace6e12c2d14e6dd569d035162aa2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516475</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786015629</t>
+          <t>1786049379</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786208400</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>19.345455</t>
+          <t>340.430769</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,23 +747,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+          <t>0x141eb383c834f2311a0a971f6b102c95bbfbe72bf5aec96515326e8a44f36f73</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.10054</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -779,7 +775,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -802,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785807147</t>
+          <t>1786048863</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>3.76253</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+          <t>0x081ed159819d5a8a466bbae50bce4afd7d1ff9c80e37e3a8963dae2b0d164087</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0525</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785805367</t>
+          <t>1786048862</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>28.761905</t>
+          <t>34.188034</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,23 +971,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0xeadb7cbd384b3086a046b663a41d256f25782ec87a602e53327804ac26f8649e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>19.0949</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0662</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -995,7 +999,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Estrela Amadora</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1003,27 +1011,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1056,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1786045554</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>288.224906</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,31 +1083,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0xbd425b3af942b740eb524c67b09d901520f7e36f781edec39fe94f990058f28e</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4937</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1122,7 +1138,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1786045527</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>6.622785</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,12 +1195,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x211e89a27cd857cfac01ad444d50285b78d7687ef94b8ec9d29ddf115e3f1b77</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1194,12 +1210,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10.12292</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2975</t>
+          <t>1.0362</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1209,7 +1225,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1219,27 +1235,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>SL Benfica FC vs Academico Viseu</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19551968</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1280,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1786045134</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786303800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>279.252966</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,27 +1307,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0xeae7a78ab89105d02d28035125423525a0f8deab5d784f8092d1eae4a21a21ae</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>20.58</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.2125</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1319,11 +1331,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1331,27 +1339,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x8240d316399f4df8430aecf2d4dff464b80ec9896c3e9a4a49cec6126730b286</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1384,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1786043934</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>96.847059</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,110 +1411,982 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1.025</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.0513</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>FC Porto vs Alverca</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19516476</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786025695</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786294800</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>7.98</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.4125</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786015629</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>19.345455</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1785807147</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1.383562</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.0525</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FC Porto vs Alverca</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19516476</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1785805367</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786294800</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>28.761905</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>70.81</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1785793268</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>97.0</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1785792146</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>1.383562</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.2975</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1785703082</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>3.361345</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-06 23:02:33 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xc6ee63bfb29ff37d865d39e8b8e92d29aa6d4569f5768aa6ccfbd9a9d9b5ea27</t>
+          <t>0xcf652ab3194f9d567f6ddf3cdd019d440a65e8947d916dc3738e0335bbd3fe07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xceeDe2b5168e0CBeCe1a33e07B384deDB5ea627A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.66</t>
+          <t>10.8425</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.0388</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>SL Benfica FC vs Academico Viseu</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19551968</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786053177</t>
+          <t>1786054302</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786303800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>11.619048</t>
+          <t>279.806452</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xeb3ffa21a81bad64e1c57daa8b3b700ccd2e0a139717709a792ed1a5fe326ca8</t>
+          <t>0xc6ee63bfb29ff37d865d39e8b8e92d29aa6d4569f5768aa6ccfbd9a9d9b5ea27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786049713</t>
+          <t>1786053177</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>11.301587</t>
+          <t>11.619048</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,23 +755,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xcbddf823e635f74877809e664d307d69fbe07274867c3fdd6f6b327d9b61cfd2</t>
+          <t>0xeb3ffa21a81bad64e1c57daa8b3b700ccd2e0a139717709a792ed1a5fe326ca8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>165.96</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4875</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -779,7 +783,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -787,27 +795,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes vs FC Arouca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>FC Arouca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x1952e4e0eea3adef3eef21ecd14324031f0ace6e12c2d14e6dd569d035162aa2</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19516475</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +840,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786049379</t>
+          <t>1786049713</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786208400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>340.430769</t>
+          <t>11.301587</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x141eb383c834f2311a0a971f6b102c95bbfbe72bf5aec96515326e8a44f36f73</t>
+          <t>0xcbddf823e635f74877809e664d307d69fbe07274867c3fdd6f6b327d9b61cfd2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -867,19 +875,15 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.10054</t>
+          <t>165.96</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2925</t>
+          <t>1.4875</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -887,11 +891,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -899,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Vitoria Guimaraes vs FC Arouca</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>FC Arouca</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0x1952e4e0eea3adef3eef21ecd14324031f0ace6e12c2d14e6dd569d035162aa2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516475</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786048863</t>
+          <t>1786049379</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786208400</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>3.76253</t>
+          <t>340.430769</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +971,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x081ed159819d5a8a466bbae50bce4afd7d1ff9c80e37e3a8963dae2b0d164087</t>
+          <t>0x141eb383c834f2311a0a971f6b102c95bbfbe72bf5aec96515326e8a44f36f73</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.10054</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786048862</t>
+          <t>1786048863</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>34.188034</t>
+          <t>3.76253</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1083,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xeadb7cbd384b3086a046b663a41d256f25782ec87a602e53327804ac26f8649e</t>
+          <t>0x081ed159819d5a8a466bbae50bce4afd7d1ff9c80e37e3a8963dae2b0d164087</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,12 +1098,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>19.0949</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.0662</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1123,27 +1123,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1168,17 +1168,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786045554</t>
+          <t>1786048862</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>288.224906</t>
+          <t>34.188034</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,12 +1195,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xbd425b3af942b740eb524c67b09d901520f7e36f781edec39fe94f990058f28e</t>
+          <t>0xeadb7cbd384b3086a046b663a41d256f25782ec87a602e53327804ac26f8649e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1210,22 +1210,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>19.0949</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4937</t>
+          <t>1.0662</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1235,27 +1235,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
+          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786045527</t>
+          <t>1786045554</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6.622785</t>
+          <t>288.224906</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1307,12 +1307,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x211e89a27cd857cfac01ad444d50285b78d7687ef94b8ec9d29ddf115e3f1b77</t>
+          <t>0xbd425b3af942b740eb524c67b09d901520f7e36f781edec39fe94f990058f28e</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1322,22 +1322,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.12292</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.0362</t>
+          <t>1.4937</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Academico Viseu</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1347,27 +1347,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>SL Benfica FC vs Academico Viseu</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Academico Viseu</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
+          <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19551968</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1392,17 +1392,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786045134</t>
+          <t>1786045527</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786303800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>279.252966</t>
+          <t>6.622785</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xeae7a78ab89105d02d28035125423525a0f8deab5d784f8092d1eae4a21a21ae</t>
+          <t>0x211e89a27cd857cfac01ad444d50285b78d7687ef94b8ec9d29ddf115e3f1b77</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1427,15 +1427,19 @@
           <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>20.58</t>
+          <t>10.12292</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2125</t>
+          <t>1.0362</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1443,7 +1447,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Academico Viseu</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1451,27 +1459,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>SL Benfica FC vs Academico Viseu</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x8240d316399f4df8430aecf2d4dff464b80ec9896c3e9a4a49cec6126730b286</t>
+          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19551968</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1504,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786043934</t>
+          <t>1786045134</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786303800</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>96.847059</t>
+          <t>279.252966</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,27 +1531,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
+          <t>0xeae7a78ab89105d02d28035125423525a0f8deab5d784f8092d1eae4a21a21ae</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>20.58</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.0513</t>
+          <t>1.2125</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1551,11 +1555,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Alverca</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1563,27 +1563,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0x8240d316399f4df8430aecf2d4dff464b80ec9896c3e9a4a49cec6126730b286</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1608,17 +1608,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786025695</t>
+          <t>1786043934</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>96.847059</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,12 +1635,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
+          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>1.025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4125</t>
+          <t>1.0513</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1675,27 +1675,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1720,17 +1720,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786015629</t>
+          <t>1786025695</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>19.345455</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1747,23 +1747,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.4125</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1771,7 +1775,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1794,7 +1802,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1832,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785807147</t>
+          <t>1786015629</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1842,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>19.345455</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1859,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1859,19 +1867,15 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.0525</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1879,11 +1883,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Alverca</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1891,27 +1891,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1936,17 +1936,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785805367</t>
+          <t>1785807147</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>28.761905</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,7 +1963,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1971,15 +1971,19 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0525</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1987,7 +1991,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1995,27 +2003,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2040,17 +2048,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1785805367</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>28.761905</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2067,7 +2075,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2078,7 +2086,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>70.81</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2144,7 +2152,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2162,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,27 +2179,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2975</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2199,11 +2203,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,12 +2283,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2298,12 +2298,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.2975</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2313,32 +2313,32 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785703082</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>3.361345</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,110 +2395,222 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 09:02:35 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
+++ b/data/sxbet/ligas/Portugal Primeira Liga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x5db545e380a7c345262ca399edfaff705347dbe69e7662421c2cefb181c038a1</t>
+          <t>0x3b1e490b754fa31393f2d7a2ac5a6643a5389c998d8b9b488402ce2e8277e440</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x7FBBAf1D0066D0f087b3686cAfd17b3B4A25Aa4b</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.07999</t>
+          <t>7.51</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6238</t>
+          <t>1.2963</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Maritimo vs Casa Pia</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Maritimo</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xca3cb5ec3b3f53dda992d93b2a2b8df8c39690bca0b23ca6da1b5951a01855b6</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19552012</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786085661</t>
+          <t>1786090860</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786199400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4.93786</t>
+          <t>25.350211</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xa0d51788e5508418113cdeaaaaabd6a1d6228c34290223cbdd343b540c546d49</t>
+          <t>0x5f3aeeada41f86405f3653b66ee344430211c2201edb7f27c69a81b507a62671</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.4537</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Portugal Primeira Liga</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FC Arouca</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes vs FC Arouca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>FC Arouca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xf17aa81af43e5328ecd75937871e6a591d9ea1f718250af6f636605eed85ea37</t>
+          <t>0x9bd57c98cbbe3e06a6f201fc351a1fb99a8ac8215e100584eaa510caf6ecfcfa</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19516475</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786082857</t>
+          <t>1786089858</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786208400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>86.956522</t>
+          <t>11.019284</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,27 +755,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x940b3d0a5f2c0d02aa00370958bd9a638dc2743fa86b198fc64dbf88b59fc4e4</t>
+          <t>0x5db545e380a7c345262ca399edfaff705347dbe69e7662421c2cefb181c038a1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x7FBBAf1D0066D0f087b3686cAfd17b3B4A25Aa4b</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.55</t>
+          <t>3.07999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.0613</t>
+          <t>1.6238</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -775,11 +779,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Estrela Amadora</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>Maritimo vs Casa Pia</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Maritimo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>Casa Pia</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
+          <t>0xca3cb5ec3b3f53dda992d93b2a2b8df8c39690bca0b23ca6da1b5951a01855b6</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19552012</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786082391</t>
+          <t>1786085661</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786199400</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>155.918367</t>
+          <t>4.93786</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd4f4471b9a4cd078621001801a4f9664ae23bf39e508c64594c0b821861ba495</t>
+          <t>0xa0d51788e5508418113cdeaaaaabd6a1d6228c34290223cbdd343b540c546d49</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0613</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>FC Arouca</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>Vitoria Guimaraes vs FC Arouca</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>FC Arouca</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
+          <t>0xf17aa81af43e5328ecd75937871e6a591d9ea1f718250af6f636605eed85ea37</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19516475</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786077443</t>
+          <t>1786082857</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786208400</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>130.612245</t>
+          <t>86.956522</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,23 +971,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x174cd45543aaf50bbbb7a07c8bd7b10d8cc42eda9c1477acb67588ce67012766</t>
+          <t>0x940b3d0a5f2c0d02aa00370958bd9a638dc2743fa86b198fc64dbf88b59fc4e4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>49.99996</t>
+          <t>9.55</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.9438</t>
+          <t>1.0613</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -995,7 +999,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Estrela Amadora</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1048,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786076636</t>
+          <t>1786082391</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>52.98009</t>
+          <t>155.918367</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,23 +1083,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x1c1eacde07c83070b93f5034bc7e9f27b7ba93e84081702d7cfc62e382a26a62</t>
+          <t>0xd4f4471b9a4cd078621001801a4f9664ae23bf39e508c64594c0b821861ba495</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>49.99996</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.9438</t>
+          <t>1.0613</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1099,7 +1111,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Estrela Amadora</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -1152,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786076571</t>
+          <t>1786077443</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>52.98009</t>
+          <t>130.612245</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x63f0ea1366c58716b1045b45e4097f32f45940128a3dafca0951a7f24fa61f80</t>
+          <t>0x174cd45543aaf50bbbb7a07c8bd7b10d8cc42eda9c1477acb67588ce67012766</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1256,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786076507</t>
+          <t>1786076636</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1283,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x4b2d4fb56a5ddac1aeba9d2899bed463f4500fc801f706f39e08458c3440cad8</t>
+          <t>0x1c1eacde07c83070b93f5034bc7e9f27b7ba93e84081702d7cfc62e382a26a62</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1360,7 +1376,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786076442</t>
+          <t>1786076571</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1387,7 +1403,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xd721a7b395e52efed2aa009849853638b368e8d8fed200f138bf826b20f8bd94</t>
+          <t>0x63f0ea1366c58716b1045b45e4097f32f45940128a3dafca0951a7f24fa61f80</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1464,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786076377</t>
+          <t>1786076507</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1491,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x457d97c5a72cfa7421cece30e9ae220d3f04c97cc6ea6fd38c666898f2ed0e04</t>
+          <t>0x4b2d4fb56a5ddac1aeba9d2899bed463f4500fc801f706f39e08458c3440cad8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1568,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786076312</t>
+          <t>1786076442</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1595,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x40348d551ffd1a398437ebe036a60b0138f6e3d3deeeee860f1cbff818e3e2c8</t>
+          <t>0xd721a7b395e52efed2aa009849853638b368e8d8fed200f138bf826b20f8bd94</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1672,7 +1688,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786076247</t>
+          <t>1786076377</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1699,7 +1715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x4f270ee3dc0a623c27e05ad5421e1236256f5e18848513e479a2f3f61b775ddf</t>
+          <t>0x457d97c5a72cfa7421cece30e9ae220d3f04c97cc6ea6fd38c666898f2ed0e04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1776,7 +1792,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786076181</t>
+          <t>1786076312</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1803,7 +1819,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x8814c112ecc59039fb893698f2b7f7260002c6bff2969a32c396a28f6d216900</t>
+          <t>0x40348d551ffd1a398437ebe036a60b0138f6e3d3deeeee860f1cbff818e3e2c8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1880,7 +1896,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786076117</t>
+          <t>1786076247</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1907,7 +1923,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xd11995b1fc2a5b6a58a93db994a16829be4aca548d22c7b34a522bb24fad8b4f</t>
+          <t>0x4f270ee3dc0a623c27e05ad5421e1236256f5e18848513e479a2f3f61b775ddf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1984,7 +2000,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786076052</t>
+          <t>1786076181</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2011,7 +2027,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xc66d09d271e30a66de590c7b1c6d5ae45ea33b28a5247c347cba16ba98528641</t>
+          <t>0x8814c112ecc59039fb893698f2b7f7260002c6bff2969a32c396a28f6d216900</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2088,7 +2104,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786075986</t>
+          <t>1786076117</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2115,7 +2131,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xdf5fd611acbffce87f7b29174db70f70571979ee615ab031a925a05d1c86f71d</t>
+          <t>0xd11995b1fc2a5b6a58a93db994a16829be4aca548d22c7b34a522bb24fad8b4f</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2126,7 +2142,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34.99996</t>
+          <t>49.99996</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2192,7 +2208,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786075410</t>
+          <t>1786076052</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2202,7 +2218,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>37.08605</t>
+          <t>52.98009</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2219,27 +2235,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x798392d3438dd61de66e0742a442cf8f3f97f7ec63181a2a338822f6427049fb</t>
+          <t>0xc66d09d271e30a66de590c7b1c6d5ae45ea33b28a5247c347cba16ba98528641</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>49.99996</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.9438</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2247,11 +2259,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -2259,27 +2267,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2304,17 +2312,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786074828</t>
+          <t>1786075986</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>9.936508</t>
+          <t>52.98009</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2331,27 +2339,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcf652ab3194f9d567f6ddf3cdd019d440a65e8947d916dc3738e0335bbd3fe07</t>
+          <t>0xdf5fd611acbffce87f7b29174db70f70571979ee615ab031a925a05d1c86f71d</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xceeDe2b5168e0CBeCe1a33e07B384deDB5ea627A</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x47d3E967E91199423245cDD504Db05a98BC30879</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.8425</t>
+          <t>34.99996</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.0388</t>
+          <t>1.9438</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2359,11 +2363,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Academico Viseu</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -2371,27 +2371,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>SL Benfica FC vs Academico Viseu</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Academico Viseu</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
+          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19551968</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2416,17 +2416,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786054302</t>
+          <t>1786075410</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786303800</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>279.806452</t>
+          <t>37.08605</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2443,7 +2443,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xc6ee63bfb29ff37d865d39e8b8e92d29aa6d4569f5768aa6ccfbd9a9d9b5ea27</t>
+          <t>0x798392d3438dd61de66e0742a442cf8f3f97f7ec63181a2a338822f6427049fb</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.66</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786053177</t>
+          <t>1786074828</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>11.619048</t>
+          <t>9.936508</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2555,12 +2555,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xeb3ffa21a81bad64e1c57daa8b3b700ccd2e0a139717709a792ed1a5fe326ca8</t>
+          <t>0xcf652ab3194f9d567f6ddf3cdd019d440a65e8947d916dc3738e0335bbd3fe07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xceeDe2b5168e0CBeCe1a33e07B384deDB5ea627A</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2570,12 +2570,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>10.8425</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.0388</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2595,27 +2595,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>SL Benfica FC vs Academico Viseu</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19551968</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2640,17 +2640,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786049713</t>
+          <t>1786054302</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786303800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>11.301587</t>
+          <t>279.806452</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,23 +2667,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xcbddf823e635f74877809e664d307d69fbe07274867c3fdd6f6b327d9b61cfd2</t>
+          <t>0xc6ee63bfb29ff37d865d39e8b8e92d29aa6d4569f5768aa6ccfbd9a9d9b5ea27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>165.96</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.4875</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2691,7 +2695,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -2699,27 +2707,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes vs FC Arouca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>FC Arouca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x1952e4e0eea3adef3eef21ecd14324031f0ace6e12c2d14e6dd569d035162aa2</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19516475</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2744,17 +2752,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786049379</t>
+          <t>1786053177</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786208400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>340.430769</t>
+          <t>11.619048</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2771,12 +2779,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x141eb383c834f2311a0a971f6b102c95bbfbe72bf5aec96515326e8a44f36f73</t>
+          <t>0xeb3ffa21a81bad64e1c57daa8b3b700ccd2e0a139717709a792ed1a5fe326ca8</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2786,12 +2794,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.10054</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.2925</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2801,7 +2809,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2826,7 +2834,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2856,7 +2864,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786048863</t>
+          <t>1786049713</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2866,7 +2874,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>3.76253</t>
+          <t>11.301587</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2883,27 +2891,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x081ed159819d5a8a466bbae50bce4afd7d1ff9c80e37e3a8963dae2b0d164087</t>
+          <t>0xcbddf823e635f74877809e664d307d69fbe07274867c3fdd6f6b327d9b61cfd2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>165.96</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2925</t>
+          <t>1.4875</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2911,11 +2915,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -2923,27 +2923,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Vitoria Guimaraes vs FC Arouca</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>FC Arouca</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0x1952e4e0eea3adef3eef21ecd14324031f0ace6e12c2d14e6dd569d035162aa2</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516475</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2968,17 +2968,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786048862</t>
+          <t>1786049379</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786208400</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>34.188034</t>
+          <t>340.430769</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2995,12 +2995,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xeadb7cbd384b3086a046b663a41d256f25782ec87a602e53327804ac26f8649e</t>
+          <t>0x141eb383c834f2311a0a971f6b102c95bbfbe72bf5aec96515326e8a44f36f73</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3010,12 +3010,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>19.0949</t>
+          <t>1.10054</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.0662</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3035,27 +3035,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3080,17 +3080,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786045554</t>
+          <t>1786048863</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>288.224906</t>
+          <t>3.76253</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xbd425b3af942b740eb524c67b09d901520f7e36f781edec39fe94f990058f28e</t>
+          <t>0x081ed159819d5a8a466bbae50bce4afd7d1ff9c80e37e3a8963dae2b0d164087</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3122,22 +3122,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4937</t>
+          <t>1.2925</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786045527</t>
+          <t>1786048862</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>6.622785</t>
+          <t>34.188034</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3219,7 +3219,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x211e89a27cd857cfac01ad444d50285b78d7687ef94b8ec9d29ddf115e3f1b77</t>
+          <t>0xeadb7cbd384b3086a046b663a41d256f25782ec87a602e53327804ac26f8649e</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3234,12 +3234,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.12292</t>
+          <t>19.0949</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.0362</t>
+          <t>1.0662</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Academico Viseu</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3259,27 +3259,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>SL Benfica FC vs Academico Viseu</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>SL Benfica FC</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Academico Viseu</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
+          <t>0x5b64345975cf00da8fa2c970c0fa395244bae67afd8a6e447359e5785d80c172</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19551968</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3304,17 +3304,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786045134</t>
+          <t>1786045554</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786303800</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>279.252966</t>
+          <t>288.224906</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3331,31 +3331,39 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xeae7a78ab89105d02d28035125423525a0f8deab5d784f8092d1eae4a21a21ae</t>
+          <t>0xbd425b3af942b740eb524c67b09d901520f7e36f781edec39fe94f990058f28e</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>20.58</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2125</t>
+          <t>1.4937</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -3363,27 +3371,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Estrela Amadora</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Sporting Clube De Portugal CP</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x8240d316399f4df8430aecf2d4dff464b80ec9896c3e9a4a49cec6126730b286</t>
+          <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19516479</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3408,17 +3416,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786043934</t>
+          <t>1786045527</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786217400</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>96.847059</t>
+          <t>6.622785</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3435,12 +3443,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
+          <t>0x211e89a27cd857cfac01ad444d50285b78d7687ef94b8ec9d29ddf115e3f1b77</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3450,12 +3458,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>10.12292</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.0513</t>
+          <t>1.0362</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3465,7 +3473,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3475,27 +3483,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>SL Benfica FC vs Academico Viseu</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>SL Benfica FC</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Academico Viseu</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0x6bd6826ca8d748573498f2ac35a20fb5c9cd65be122b2d6bd4c3445f7d1f4f28</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19551968</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3520,17 +3528,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786025695</t>
+          <t>1786045134</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786303800</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>279.252966</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3547,27 +3555,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
+          <t>0xeae7a78ab89105d02d28035125423525a0f8deab5d784f8092d1eae4a21a21ae</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>20.58</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.4125</t>
+          <t>1.2125</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3575,11 +3579,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -3587,27 +3587,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>Estrela Amadora vs Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Estrela Amadora</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Sporting Clube De Portugal CP</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0x8240d316399f4df8430aecf2d4dff464b80ec9896c3e9a4a49cec6126730b286</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516479</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3632,17 +3632,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786015629</t>
+          <t>1786043934</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786217400</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>19.345455</t>
+          <t>96.847059</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3659,23 +3659,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
+          <t>0x852ebe5fa56685e97646816bda03a75daa7be5c686a0c21e6cc91fe9e929156e</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>0xA31bC6F3C5514Cc3638BE835d196AF34aB1A8A05</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.025</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0513</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3683,7 +3687,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -3691,27 +3699,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3736,17 +3744,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785807147</t>
+          <t>1786025695</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3763,12 +3771,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
+          <t>0xfd9767efb72afaa140473f61906b464a888f1ccd0ce66296246c5feef22df0b4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3778,12 +3786,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.0525</t>
+          <t>1.4125</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3793,7 +3801,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3803,27 +3811,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>FC Porto vs Alverca</t>
+          <t>Estoril vs Famalicão</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>FC Porto</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Famalicão</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19516476</t>
+          <t>L19516436</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3848,17 +3856,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785805367</t>
+          <t>1786015629</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1786294800</t>
+          <t>1786130100</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>28.761905</t>
+          <t>19.345455</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3875,7 +3883,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
+          <t>0xe1e981f73c1f5dcbea6fbe8985aac20970e24227fdd1722c2cabaf5ab34d5ffc</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3886,7 +3894,7 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>70.81</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3952,7 +3960,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785793268</t>
+          <t>1785807147</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3962,7 +3970,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3979,7 +3987,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
+          <t>0x86326082a40b8bd83786ee356714d61b0536794f55892123cc41ac2b3f486a09</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3987,15 +3995,19 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.0525</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4003,7 +4015,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -4011,27 +4027,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Estoril vs Famalicão</t>
+          <t>FC Porto vs Alverca</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>FC Porto</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Famalicão</t>
+          <t>Alverca</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
+          <t>0xdbac9a0b5328bd2f4a2e48e69be0724e79bc4a0ce6688099035cf63f6959d637</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19516436</t>
+          <t>L19516476</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4056,17 +4072,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785792146</t>
+          <t>1785805367</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1786130100</t>
+          <t>1786294800</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1.383562</t>
+          <t>28.761905</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4083,27 +4099,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+          <t>0x3cfe50f74987860a9991087809d398727832f523a8592e4f716592807d1fcbcd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>70.81</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.2975</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4111,11 +4123,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
@@ -4138,7 +4146,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4168,7 +4176,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785703082</t>
+          <t>1785793268</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4178,7 +4186,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>3.361345</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4195,27 +4203,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+          <t>0x091493eaabf18416d304e2afc51faef0752c61a5378ff4fde277854b3aca3087</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.4512</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4223,34 +4227,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Portugal Primeira Liga</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Estoril vs Famalicão</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Estoril</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Famalicão</t>
-        </is>
-      </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+          <t>0xd90f3a9796440faedb803c6686c8d8937f0ec27180a46805e5823a336f2caa7a</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785702973</t>
+          <t>1785792146</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>3.168975</t>
+          <t>1.383562</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4307,110 +4307,334 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>0x6bd1b754d66093d507837af84d3bc61208561ca7bee41d496c52f24993630ac8</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x048c07Af144F98F1c44E64455c69Cd7343116B71</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.2975</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x78d24a131bd50c9b54c26ebb579e3b5de696381c306e9696bdd139fe355424fa</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1785703082</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>3.361345</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0xbdb9c4454911d572e7daeae99f63956fc8a2f1036f88447c7a3be966b25dcfda</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Portugal Primeira Liga</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Estoril vs Famalicão</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Famalicão</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xd1f6ef28397cea5e0fd8d621b5ffd5c7facb1e496cf5dffa97e30b23bb7ed538</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19516436</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1785702973</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786130100</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>3.168975</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>0x25c79ef1a4efff81c8eacc6dd6166f75a9278fa2138727c677760b0010164ef9</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>1.5225</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>Portugal Primeira Liga</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Estoril vs Famalicão</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Estoril</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Famalicão</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>0x9928b6bf8cc196b9ef01e3d9935c418fd4ad023101bb76da4283e20916b1a22d</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>L19516436</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>1785701935</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>1786130100</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>1.913876</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>